<commit_message>
data: retrain RECT_planar (+ export JSON) after neighborhood fix
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_results.xlsx
+++ b/outputs/metrics/model_comparison_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,40 +436,55 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>lattice</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>ARI</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>NMI</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Silhouette</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Davies-Bouldin</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Calinski-Harabasz</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Pureza Neurônios</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Erro Quantização</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Erro Topográfico</t>
         </is>
@@ -478,288 +493,1266 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SOM 5x5</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.6584356954057571</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.8063085351824245</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.1547883509123739</v>
+          <t>SOM 5x5 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>1.713133149489485</v>
+        <v>0.5989288152472451</v>
       </c>
       <c r="F2" t="n">
-        <v>177.5235309684164</v>
+        <v>0.7596573109307793</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9193008019234434</v>
+        <v>0.1396989480456421</v>
       </c>
       <c r="H2" t="n">
-        <v>4.734787500820725</v>
+        <v>1.775014507787715</v>
       </c>
       <c r="I2" t="n">
-        <v>0.24</v>
+        <v>181.5625045590118</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.8896982656379243</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.075</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SOM 7x7</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.6095062500422831</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.7550727454605211</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.1875718442552337</v>
+          <t>SOM 5x5 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>1.581399796468479</v>
+        <v>0.7708612487301378</v>
       </c>
       <c r="F3" t="n">
-        <v>204.7898015872679</v>
+        <v>0.8551548004733603</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9298783130610627</v>
+        <v>0.1458893839682167</v>
       </c>
       <c r="H3" t="n">
-        <v>4.244013158022346</v>
+        <v>1.919421297526019</v>
       </c>
       <c r="I3" t="n">
-        <v>0.12</v>
+        <v>179.9631854386272</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.9180918506755177</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.105</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SOM 10x10</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.6337364043591162</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.7713090236359282</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.2042384399548178</v>
+          <t>SOM 5x5 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>1.59749423678315</v>
+        <v>0.618191365816935</v>
       </c>
       <c r="F4" t="n">
-        <v>208.1051582559295</v>
+        <v>0.8023936573668673</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9593867243867246</v>
+        <v>0.240116284019057</v>
       </c>
       <c r="H4" t="n">
-        <v>3.903502961882596</v>
+        <v>1.224288633631303</v>
       </c>
       <c r="I4" t="n">
-        <v>0.15</v>
+        <v>203.3241927174201</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.904850514423625</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.003333333333333334</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SOM 12x12</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.6312659442034516</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.769202516686885</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.2009276747778873</v>
+          <t>SOM 5x5 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>1.602735273864879</v>
+        <v>0.6678916171098431</v>
       </c>
       <c r="F5" t="n">
-        <v>208.3848683620924</v>
+        <v>0.8229795483555994</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9899584076054664</v>
+        <v>0.0388754745487815</v>
       </c>
       <c r="H5" t="n">
-        <v>3.751180930932599</v>
+        <v>1.707725052222677</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1483333333333333</v>
+        <v>152.7802354039756</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.8955643760613194</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.03666666666666667</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SOM 15x15</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.6217376431516455</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.7625355888560764</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.2040054319515413</v>
+          <t>SOM 7x7 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>1.606272231027173</v>
+        <v>0.6149895406286217</v>
       </c>
       <c r="F6" t="n">
-        <v>209.6545098674629</v>
+        <v>0.7578906964441489</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9874485596707819</v>
+        <v>0.1964154809661962</v>
       </c>
       <c r="H6" t="n">
-        <v>3.555548621462714</v>
+        <v>1.575761081937952</v>
       </c>
       <c r="I6" t="n">
-        <v>0.065</v>
+        <v>208.3730987530203</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.9213449655674334</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SOM 20x20</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.5878776276859684</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.7591249096233086</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.2629194315953705</v>
+          <t>SOM 7x7 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
       </c>
       <c r="E7" t="n">
-        <v>1.207375846233864</v>
+        <v>0.6559087103624082</v>
       </c>
       <c r="F7" t="n">
-        <v>213.2737780890826</v>
+        <v>0.7926104574035003</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9967320261437909</v>
+        <v>0.1995239121760161</v>
       </c>
       <c r="H7" t="n">
-        <v>3.334735347915241</v>
+        <v>1.559953766047531</v>
       </c>
       <c r="I7" t="n">
-        <v>0.045</v>
+        <v>206.5479351054552</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9451590966965298</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.01833333333333333</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>K-Means (Direto)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.568100291666193</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.7410812863322819</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.2710398322948481</v>
+          <t>SOM 7x7 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
       </c>
       <c r="E8" t="n">
-        <v>1.210505956597288</v>
+        <v>0.6124609113218785</v>
       </c>
       <c r="F8" t="n">
-        <v>214.486932345493</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+        <v>0.7726085528091295</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.176545059498681</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.59442923835971</v>
+      </c>
+      <c r="I8" t="n">
+        <v>194.1007168862327</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.9404592741280048</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.015</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PCA + K-Means</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.6096211462315787</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.7188561117363224</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.1481066860982583</v>
+          <t>SOM 7x7 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
       </c>
       <c r="E9" t="n">
-        <v>1.950508371568407</v>
+        <v>0.5433195879666382</v>
       </c>
       <c r="F9" t="n">
-        <v>182.7762443503514</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+        <v>0.7116216992564081</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1512098933716221</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.889379324798274</v>
+      </c>
+      <c r="I9" t="n">
+        <v>187.1537030622428</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.9449611229390641</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.04833333333333333</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Agglomerative (K=6)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.616042904903928</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.8007911127058996</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.250993518422146</v>
+          <t>SOM 10x10 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
       </c>
       <c r="E10" t="n">
-        <v>1.202078390062834</v>
+        <v>0.6385170139974198</v>
       </c>
       <c r="F10" t="n">
-        <v>209.5237290780118</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+        <v>0.7849491803602441</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.2029285092326681</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.616244232669046</v>
+      </c>
+      <c r="I10" t="n">
+        <v>205.6385272701472</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.9510476190476191</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.07333333333333333</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>SOM 10x10 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.6607868032366434</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.7975337572164257</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.2049238515860173</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.556312094909461</v>
+      </c>
+      <c r="I11" t="n">
+        <v>210.2275956388356</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.01166666666666667</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SOM 10x10 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.6110597423308181</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7912213064948445</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.2497882568396752</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.213888174827302</v>
+      </c>
+      <c r="I12" t="n">
+        <v>209.0514424922801</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.9850210970464135</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.001666666666666667</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SOM 10x10 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.63179016073248</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7659238581453671</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.2081070185574844</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.606499520771478</v>
+      </c>
+      <c r="I13" t="n">
+        <v>209.8385527690805</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.9661349911349911</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SOM 12x12 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.6321338159747251</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.7749631936461956</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2008382240817951</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1.584546053640502</v>
+      </c>
+      <c r="I14" t="n">
+        <v>209.0683934036545</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.9775891874901775</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.05333333333333334</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SOM 12x12 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.6079393509292708</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.7837338428813686</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.2525359242572511</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.21238865675846</v>
+      </c>
+      <c r="I15" t="n">
+        <v>208.3165354930798</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.9878260869565217</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.003333333333333334</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SOM 12x12 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.6689707022385961</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.8034922360293735</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.2017700426087989</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.556761190811165</v>
+      </c>
+      <c r="I16" t="n">
+        <v>207.3488663062654</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.9875541125541125</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.006666666666666667</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SOM 12x12 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.693987585712084</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.8271456389924026</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.2048920663490574</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1.559373428782702</v>
+      </c>
+      <c r="I17" t="n">
+        <v>209.7503579598541</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.9794238683127572</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SOM 15x15 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.5875010961305213</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.7577491012263263</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.2624814244925067</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1.205698756906799</v>
+      </c>
+      <c r="I18" t="n">
+        <v>212.9783136270856</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.9877358490566038</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.02166666666666667</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SOM 15x15 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.5905426187976452</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.7614982302245642</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.2607447671779279</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.210479692289825</v>
+      </c>
+      <c r="I19" t="n">
+        <v>211.8779583077049</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.9890476190476191</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.006666666666666667</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SOM 15x15 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.6481798657021782</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.7885670188082193</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.2046974682360846</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.61029454422935</v>
+      </c>
+      <c r="I20" t="n">
+        <v>208.8059159426398</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.9872549019607844</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SOM 15x15 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.6494566538074247</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.7929354742399427</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.2027385576924651</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.613666094331541</v>
+      </c>
+      <c r="I21" t="n">
+        <v>208.2989683425557</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.9905228758169935</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.02833333333333333</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SOM 20x20 HEX_toroid</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HEX_toroid</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.58706507025057</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.7617861903058081</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.2644704989132871</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.205644687564481</v>
+      </c>
+      <c r="I22" t="n">
+        <v>213.5862475227191</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.9924528301886792</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.02666666666666667</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SOM 20x20 HEX_planar</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HEX</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>HEX_planar</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.6582081391792047</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8006438106341009</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.2039291221850801</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.609292594903254</v>
+      </c>
+      <c r="I23" t="n">
+        <v>206.8426273827262</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.9950433705080544</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.01166666666666667</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SOM 20x20 RECT_planar</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>planar</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RECT_planar</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.6617177967424988</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.7996817204412167</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.2039383363917057</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.550444781573064</v>
+      </c>
+      <c r="I24" t="n">
+        <v>210.2443264946179</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.9949874686716791</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.003333333333333334</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SOM 20x20 RECT_toroid</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>toroid</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RECT_toroid</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.6660664371613503</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.7989498871415586</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.2039371823408551</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.546701414119193</v>
+      </c>
+      <c r="I25" t="n">
+        <v>210.1266592310527</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.981908302354399</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.02666666666666667</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>K-Means (Direto)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.568100291666193</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.7410812863322819</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.2710398322948481</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.210505956597288</v>
+      </c>
+      <c r="I26" t="n">
+        <v>214.486932345493</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PCA + K-Means</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.6096211462315787</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.7188561117363224</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.1481066860982583</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.950508371568407</v>
+      </c>
+      <c r="I27" t="n">
+        <v>182.7762443503514</v>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Agglomerative (K=6)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.616042904903928</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.8007911127058996</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.250993518422146</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.202078390062834</v>
+      </c>
+      <c r="I28" t="n">
+        <v>209.5237290780118</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>DBSCAN</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
         <v>0.1418338108882521</v>
       </c>
-      <c r="C11" t="n">
+      <c r="F29" t="n">
         <v>0.40187044901108</v>
       </c>
-      <c r="D11" t="n">
+      <c r="G29" t="n">
         <v>0.1818959068791801</v>
       </c>
-      <c r="E11" t="n">
+      <c r="H29" t="n">
         <v>2.349495177792563</v>
       </c>
-      <c r="F11" t="n">
+      <c r="I29" t="n">
         <v>55.96402879163693</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(metrics): recompute QE manually after load_som (property not refreshed on reload)
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_results.xlsx
+++ b/outputs/metrics/model_comparison_results.xlsx
@@ -512,25 +512,25 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5989288152472451</v>
+        <v>0.5910111920696967</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7596573109307793</v>
+        <v>0.7580228844702114</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1396989480456421</v>
+        <v>0.1519232148694801</v>
       </c>
       <c r="H2" t="n">
-        <v>1.775014507787715</v>
+        <v>1.820091933874654</v>
       </c>
       <c r="I2" t="n">
-        <v>181.5625045590118</v>
+        <v>184.625663479612</v>
       </c>
       <c r="J2" t="n">
         <v>0.8896982656379243</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>4.74019308042447</v>
       </c>
       <c r="L2" t="n">
         <v>0.075</v>
@@ -558,25 +558,25 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.7708612487301378</v>
+        <v>0.5966443613805447</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8551548004733603</v>
+        <v>0.7504202298756517</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1458893839682167</v>
+        <v>0.1905801778638978</v>
       </c>
       <c r="H3" t="n">
-        <v>1.919421297526019</v>
+        <v>1.593019805600868</v>
       </c>
       <c r="I3" t="n">
-        <v>179.9631854386272</v>
+        <v>202.1735147779932</v>
       </c>
       <c r="J3" t="n">
         <v>0.9180918506755177</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>4.335419775743943</v>
       </c>
       <c r="L3" t="n">
         <v>0.105</v>
@@ -604,25 +604,25 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.618191365816935</v>
+        <v>0.6317937786897571</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8023936573668673</v>
+        <v>0.8150071733886569</v>
       </c>
       <c r="G4" t="n">
-        <v>0.240116284019057</v>
+        <v>0.1473109768085794</v>
       </c>
       <c r="H4" t="n">
-        <v>1.224288633631303</v>
+        <v>1.607894236605629</v>
       </c>
       <c r="I4" t="n">
-        <v>203.3241927174201</v>
+        <v>187.0385272796511</v>
       </c>
       <c r="J4" t="n">
         <v>0.904850514423625</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>4.308238896711789</v>
       </c>
       <c r="L4" t="n">
         <v>0.003333333333333334</v>
@@ -650,25 +650,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.6678916171098431</v>
+        <v>0.6674087975971612</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8229795483555994</v>
+        <v>0.8279566221641198</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0388754745487815</v>
+        <v>0.07980698595556596</v>
       </c>
       <c r="H5" t="n">
-        <v>1.707725052222677</v>
+        <v>2.44774675562121</v>
       </c>
       <c r="I5" t="n">
-        <v>152.7802354039756</v>
+        <v>153.3355583778489</v>
       </c>
       <c r="J5" t="n">
         <v>0.8955643760613194</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>4.933731317248552</v>
       </c>
       <c r="L5" t="n">
         <v>0.03666666666666667</v>
@@ -696,25 +696,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.6149895406286217</v>
+        <v>0.6300372026809072</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7578906964441489</v>
+        <v>0.7767412853179155</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1964154809661962</v>
+        <v>0.1993234223939499</v>
       </c>
       <c r="H6" t="n">
-        <v>1.575761081937952</v>
+        <v>1.573161132498757</v>
       </c>
       <c r="I6" t="n">
-        <v>208.3730987530203</v>
+        <v>209.3507631067368</v>
       </c>
       <c r="J6" t="n">
         <v>0.9213449655674334</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>4.282088126870838</v>
       </c>
       <c r="L6" t="n">
         <v>0.11</v>
@@ -742,25 +742,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6559087103624082</v>
+        <v>0.6144894831201347</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7926104574035003</v>
+        <v>0.7562161084247047</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1995239121760161</v>
+        <v>0.2097073520636526</v>
       </c>
       <c r="H7" t="n">
-        <v>1.559953766047531</v>
+        <v>1.576539269272724</v>
       </c>
       <c r="I7" t="n">
-        <v>206.5479351054552</v>
+        <v>207.0022503500522</v>
       </c>
       <c r="J7" t="n">
         <v>0.9451590966965298</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>4.017378004912145</v>
       </c>
       <c r="L7" t="n">
         <v>0.01833333333333333</v>
@@ -788,25 +788,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.6124609113218785</v>
+        <v>0.6122413224268071</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7726085528091295</v>
+        <v>0.7670252808925565</v>
       </c>
       <c r="G8" t="n">
-        <v>0.176545059498681</v>
+        <v>0.1854642033613371</v>
       </c>
       <c r="H8" t="n">
-        <v>1.59442923835971</v>
+        <v>1.639334879220348</v>
       </c>
       <c r="I8" t="n">
-        <v>194.1007168862327</v>
+        <v>196.2288885124557</v>
       </c>
       <c r="J8" t="n">
         <v>0.9404592741280048</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>4.057223534886933</v>
       </c>
       <c r="L8" t="n">
         <v>0.015</v>
@@ -834,25 +834,25 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.5433195879666382</v>
+        <v>0.6339809522594915</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7116216992564081</v>
+        <v>0.7639667291998733</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1512098933716221</v>
+        <v>0.07366596871351438</v>
       </c>
       <c r="H9" t="n">
-        <v>1.889379324798274</v>
+        <v>2.377005251708499</v>
       </c>
       <c r="I9" t="n">
-        <v>187.1537030622428</v>
+        <v>160.1486744501652</v>
       </c>
       <c r="J9" t="n">
         <v>0.9449611229390641</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>4.349351431572176</v>
       </c>
       <c r="L9" t="n">
         <v>0.04833333333333333</v>
@@ -880,25 +880,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.6385170139974198</v>
+        <v>0.6405220352282578</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7849491803602441</v>
+        <v>0.7979667124289401</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2029285092326681</v>
+        <v>0.1945712341633376</v>
       </c>
       <c r="H10" t="n">
-        <v>1.616244232669046</v>
+        <v>1.579721540450318</v>
       </c>
       <c r="I10" t="n">
-        <v>205.6385272701472</v>
+        <v>205.8003734994815</v>
       </c>
       <c r="J10" t="n">
         <v>0.9510476190476191</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>3.898889076770459</v>
       </c>
       <c r="L10" t="n">
         <v>0.07333333333333333</v>
@@ -926,25 +926,25 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.6607868032366434</v>
+        <v>0.6630151754239914</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7975337572164257</v>
+        <v>0.7982980727123169</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2049238515860173</v>
+        <v>0.2025503407404985</v>
       </c>
       <c r="H11" t="n">
-        <v>1.556312094909461</v>
+        <v>1.553153978140701</v>
       </c>
       <c r="I11" t="n">
-        <v>210.2275956388356</v>
+        <v>207.7952775429848</v>
       </c>
       <c r="J11" t="n">
         <v>0.97</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>3.762781963280438</v>
       </c>
       <c r="L11" t="n">
         <v>0.01166666666666667</v>
@@ -972,25 +972,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.6110597423308181</v>
+        <v>0.6718906788660898</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7912213064948445</v>
+        <v>0.8107427826462223</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2497882568396752</v>
+        <v>0.2039224004504417</v>
       </c>
       <c r="H12" t="n">
-        <v>1.213888174827302</v>
+        <v>1.617308673766989</v>
       </c>
       <c r="I12" t="n">
-        <v>209.0514424922801</v>
+        <v>206.5961828845756</v>
       </c>
       <c r="J12" t="n">
         <v>0.9850210970464135</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>3.711782082154734</v>
       </c>
       <c r="L12" t="n">
         <v>0.001666666666666667</v>
@@ -1018,25 +1018,25 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.63179016073248</v>
+        <v>0.5852144077868013</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7659238581453671</v>
+        <v>0.7436142875988111</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2081070185574844</v>
+        <v>0.1753735744633963</v>
       </c>
       <c r="H13" t="n">
-        <v>1.606499520771478</v>
+        <v>1.628604786570839</v>
       </c>
       <c r="I13" t="n">
-        <v>209.8385527690805</v>
+        <v>200.402710211905</v>
       </c>
       <c r="J13" t="n">
         <v>0.9661349911349911</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>3.914259298799631</v>
       </c>
       <c r="L13" t="n">
         <v>0.07000000000000001</v>
@@ -1064,25 +1064,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.6321338159747251</v>
+        <v>0.6541629590078119</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7749631936461956</v>
+        <v>0.8017219597558398</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2008382240817951</v>
+        <v>0.2081443698219537</v>
       </c>
       <c r="H14" t="n">
-        <v>1.584546053640502</v>
+        <v>1.587322981225553</v>
       </c>
       <c r="I14" t="n">
-        <v>209.0683934036545</v>
+        <v>207.1177365044352</v>
       </c>
       <c r="J14" t="n">
         <v>0.9775891874901775</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>3.732294135968332</v>
       </c>
       <c r="L14" t="n">
         <v>0.05333333333333334</v>
@@ -1110,25 +1110,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.6079393509292708</v>
+        <v>0.65883041256467</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7837338428813686</v>
+        <v>0.7941374163852586</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2525359242572511</v>
+        <v>0.2071096900654809</v>
       </c>
       <c r="H15" t="n">
-        <v>1.21238865675846</v>
+        <v>1.559156053351054</v>
       </c>
       <c r="I15" t="n">
-        <v>208.3165354930798</v>
+        <v>209.0183309862515</v>
       </c>
       <c r="J15" t="n">
         <v>0.9878260869565217</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>3.612777580571731</v>
       </c>
       <c r="L15" t="n">
         <v>0.003333333333333334</v>
@@ -1156,25 +1156,25 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.6689707022385961</v>
+        <v>0.597034436175874</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8034922360293735</v>
+        <v>0.7693906306712307</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2017700426087989</v>
+        <v>0.2589721085148076</v>
       </c>
       <c r="H16" t="n">
-        <v>1.556761190811165</v>
+        <v>1.205479697689291</v>
       </c>
       <c r="I16" t="n">
-        <v>207.3488663062654</v>
+        <v>212.2699629457159</v>
       </c>
       <c r="J16" t="n">
         <v>0.9875541125541125</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3.594967650287345</v>
       </c>
       <c r="L16" t="n">
         <v>0.006666666666666667</v>
@@ -1202,25 +1202,25 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.693987585712084</v>
+        <v>0.6040024337071833</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8271456389924026</v>
+        <v>0.7591674484419968</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2048920663490574</v>
+        <v>0.196658825183823</v>
       </c>
       <c r="H17" t="n">
-        <v>1.559373428782702</v>
+        <v>1.623339174697039</v>
       </c>
       <c r="I17" t="n">
-        <v>209.7503579598541</v>
+        <v>206.0559673235233</v>
       </c>
       <c r="J17" t="n">
         <v>0.9794238683127572</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>3.736811397060534</v>
       </c>
       <c r="L17" t="n">
         <v>0.05</v>
@@ -1248,25 +1248,25 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.5875010961305213</v>
+        <v>0.641931307693025</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7577491012263263</v>
+        <v>0.7794771706707166</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2624814244925067</v>
+        <v>0.2047633786869598</v>
       </c>
       <c r="H18" t="n">
-        <v>1.205698756906799</v>
+        <v>1.562669873350209</v>
       </c>
       <c r="I18" t="n">
-        <v>212.9783136270856</v>
+        <v>210.3038979162485</v>
       </c>
       <c r="J18" t="n">
         <v>0.9877358490566038</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>3.512992934544517</v>
       </c>
       <c r="L18" t="n">
         <v>0.02166666666666667</v>
@@ -1294,25 +1294,25 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.5905426187976452</v>
+        <v>0.5901601461460088</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7614982302245642</v>
+        <v>0.7612542501445383</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2607447671779279</v>
+        <v>0.2618096364317686</v>
       </c>
       <c r="H19" t="n">
-        <v>1.210479692289825</v>
+        <v>1.202765254015002</v>
       </c>
       <c r="I19" t="n">
-        <v>211.8779583077049</v>
+        <v>212.956206937195</v>
       </c>
       <c r="J19" t="n">
         <v>0.9890476190476191</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>3.425026189204773</v>
       </c>
       <c r="L19" t="n">
         <v>0.006666666666666667</v>
@@ -1340,25 +1340,25 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.6481798657021782</v>
+        <v>0.5980764334801167</v>
       </c>
       <c r="F20" t="n">
-        <v>0.7885670188082193</v>
+        <v>0.7763724876163457</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2046974682360846</v>
+        <v>0.2583541375575693</v>
       </c>
       <c r="H20" t="n">
-        <v>1.61029454422935</v>
+        <v>1.215690882128577</v>
       </c>
       <c r="I20" t="n">
-        <v>208.8059159426398</v>
+        <v>211.9457540677187</v>
       </c>
       <c r="J20" t="n">
         <v>0.9872549019607844</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>3.458349600784816</v>
       </c>
       <c r="L20" t="n">
         <v>0.005</v>
@@ -1386,25 +1386,25 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.6494566538074247</v>
+        <v>0.6533427412372508</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7929354742399427</v>
+        <v>0.7913033665070951</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2027385576924651</v>
+        <v>0.2057325939960717</v>
       </c>
       <c r="H21" t="n">
-        <v>1.613666094331541</v>
+        <v>1.609032089553208</v>
       </c>
       <c r="I21" t="n">
-        <v>208.2989683425557</v>
+        <v>208.815291246083</v>
       </c>
       <c r="J21" t="n">
         <v>0.9905228758169935</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>3.546431731067405</v>
       </c>
       <c r="L21" t="n">
         <v>0.02833333333333333</v>
@@ -1432,25 +1432,25 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.58706507025057</v>
+        <v>0.6571436105198851</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7617861903058081</v>
+        <v>0.7886841821383326</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2644704989132871</v>
+        <v>0.2049953618613949</v>
       </c>
       <c r="H22" t="n">
-        <v>1.205644687564481</v>
+        <v>1.55671150240231</v>
       </c>
       <c r="I22" t="n">
-        <v>213.5862475227191</v>
+        <v>210.5588209664569</v>
       </c>
       <c r="J22" t="n">
         <v>0.9924528301886792</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>3.319641756639976</v>
       </c>
       <c r="L22" t="n">
         <v>0.02666666666666667</v>
@@ -1478,25 +1478,25 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.6582081391792047</v>
+        <v>0.5925586561355913</v>
       </c>
       <c r="F23" t="n">
-        <v>0.8006438106341009</v>
+        <v>0.7675359246863851</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2039291221850801</v>
+        <v>0.2586889442302066</v>
       </c>
       <c r="H23" t="n">
-        <v>1.609292594903254</v>
+        <v>1.214922830180119</v>
       </c>
       <c r="I23" t="n">
-        <v>206.8426273827262</v>
+        <v>211.8356221702341</v>
       </c>
       <c r="J23" t="n">
         <v>0.9950433705080544</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>3.235728054832324</v>
       </c>
       <c r="L23" t="n">
         <v>0.01166666666666667</v>
@@ -1524,25 +1524,25 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.6617177967424988</v>
+        <v>0.6594240029084679</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7996817204412167</v>
+        <v>0.7979988123099477</v>
       </c>
       <c r="G24" t="n">
-        <v>0.2039383363917057</v>
+        <v>0.2043367077382683</v>
       </c>
       <c r="H24" t="n">
-        <v>1.550444781573064</v>
+        <v>1.60096080333698</v>
       </c>
       <c r="I24" t="n">
-        <v>210.2443264946179</v>
+        <v>207.7719495033821</v>
       </c>
       <c r="J24" t="n">
         <v>0.9949874686716791</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>3.242026040344519</v>
       </c>
       <c r="L24" t="n">
         <v>0.003333333333333334</v>
@@ -1570,25 +1570,25 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.6660664371613503</v>
+        <v>0.6506651878175282</v>
       </c>
       <c r="F25" t="n">
-        <v>0.7989498871415586</v>
+        <v>0.7892589946496136</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2039371823408551</v>
+        <v>0.2052831947404045</v>
       </c>
       <c r="H25" t="n">
-        <v>1.546701414119193</v>
+        <v>1.542747099701429</v>
       </c>
       <c r="I25" t="n">
-        <v>210.1266592310527</v>
+        <v>211.2770447163117</v>
       </c>
       <c r="J25" t="n">
         <v>0.981908302354399</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>3.319156012901747</v>
       </c>
       <c r="L25" t="n">
         <v>0.02666666666666667</v>

</xml_diff>